<commit_message>
update: clean up files
</commit_message>
<xml_diff>
--- a/Competencies/01. Professional Skills & Manage and Control/logboek.xlsx
+++ b/Competencies/01. Professional Skills & Manage and Control/logboek.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Totaal gewerkte uren:</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>testen als mij plan van aanpak ook in realitijd werkt</t>
+  </si>
+  <si>
+    <t>De feedback van mijn docent over de folderstructuur heb ik verwerkt in mijn documentatie. Daarnaast heb ik mijn document aangepast, zodat ik meer focus leg op het proces en minder op wat ik heb geleerd.</t>
+  </si>
+  <si>
+    <t>De Tutti app is verder ontwikkeld en uitgebreid met OPAS-data en documentintegratie via SharePoint. Daarnaast zijn de beveiliging, foutafhandeling en downloads verbeterd en is de app uitgebreid getest.</t>
   </si>
 </sst>
 </file>
@@ -681,7 +687,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -689,6 +695,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1063,7 +1072,7 @@
       </c>
       <c r="B1">
         <f>SUM(B5:B1000)</f>
-        <v>40</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1072,7 +1081,7 @@
       </c>
       <c r="B2">
         <f>COUNTA(A5:A1000)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1147,17 +1156,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
+    <row r="11" ht="90" spans="1:4">
+      <c r="A11" s="3">
+        <v>46290</v>
+      </c>
+      <c r="B11" s="4">
+        <v>8</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" ht="105" spans="1:4">
+      <c r="A13" s="3">
+        <v>46295</v>
+      </c>
+      <c r="B13" s="4">
+        <v>8</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="3"/>

</xml_diff>